<commit_message>
docs(feature-report): mark #49 / #50 / #68 LIVE post-build
- #49 Supplement Stack Recommendations: PLANNED → LIVE
  (recommend-supplements endpoint + SupplementStack component)
- #50 Recovery Protocol Engine: PLANNED → LIVE
  (recovery-readout endpoint + RecoveryReadout panel)
- #68 Bilingual Voice Comms: tightened description — full app
  translation (142 keys/lang) with persistence + auto-detect, not
  just Gunny acks
- #46 Custom Video Upload + #47 AI Form Analysis (Video): explicit
  "DEFERRED next session" tag (photo form analysis remains LIVE)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/GUNS_UP_Feature_Report.xlsx
+++ b/docs/GUNS_UP_Feature_Report.xlsx
@@ -188,7 +188,7 @@
       <color rgb="00FFB800"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -231,6 +231,16 @@
         <bgColor rgb="FF0A0A0A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8F7C8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4B5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -266,7 +276,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -433,6 +443,12 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -702,7 +718,7 @@
     <row r="1" ht="19.7" customHeight="1" s="29">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>Generated April 27, 2026 (post-audit) — replaces March 23, 2026 version</t>
+          <t>Generated April 26, 2026 (post-build) — replaces April 27 audit version</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2125,7 @@
           <t>Workout</t>
         </is>
       </c>
-      <c r="D50" s="40" t="inlineStr">
+      <c r="D50" s="58" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
@@ -2121,7 +2137,7 @@
       </c>
       <c r="F50" s="38" t="inlineStr">
         <is>
-          <t>Record personal form videos during workouts → save to library</t>
+          <t>DEFERRED: Record personal form videos during workouts → save to library. Spec written, next session implementation. Targeting OPERATOR+ tier.</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2147,7 @@
       </c>
       <c r="B51" s="34" t="inlineStr">
         <is>
-          <t>AI Form Analysis</t>
+          <t>AI Form Analysis (Video)</t>
         </is>
       </c>
       <c r="C51" s="35" t="inlineStr">
@@ -2139,7 +2155,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="D51" s="40" t="inlineStr">
+      <c r="D51" s="58" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
@@ -2151,7 +2167,7 @@
       </c>
       <c r="F51" s="38" t="inlineStr">
         <is>
-          <t>Video analysis of exercise form with corrections</t>
+          <t>DEFERRED: Multi-frame video form analysis — corrections frame-by-frame. Photo Form Analysis (single image input) already LIVE via /api/gunny/analyze-form. Next session.</t>
         </is>
       </c>
     </row>
@@ -2199,9 +2215,9 @@
           <t>Nutrition</t>
         </is>
       </c>
-      <c r="D53" s="40" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="D53" s="59" t="inlineStr">
+        <is>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="E53" s="37" t="inlineStr">
@@ -2211,7 +2227,7 @@
       </c>
       <c r="F53" s="38" t="inlineStr">
         <is>
-          <t>AI-driven supplement suggestions based on goals</t>
+          <t>Evidence-based supplement stack engine (POST /api/gunny/recommend-supplements). Whitelist: creatine, whey, casein, vitamin D, magnesium glycinate, omega-3, caffeine, beta-alanine, citrulline. Rejects snake oil (BCAAs, mass gainers, T-boosters, fat burners). Hard refusals: junior operators, eating-disorder/RED-S flags, pregnancy. Rendered in IntelCenter NUTRITION tab via SupplementStack component, persists on operator.nutrition.supplementStack.</t>
         </is>
       </c>
     </row>
@@ -2229,9 +2245,9 @@
           <t>Wearable</t>
         </is>
       </c>
-      <c r="D54" s="40" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="D54" s="59" t="inlineStr">
+        <is>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="E54" s="37" t="inlineStr">
@@ -2241,7 +2257,7 @@
       </c>
       <c r="F54" s="38" t="inlineStr">
         <is>
-          <t>Auto-adjust training based on HRV/sleep data</t>
+          <t>Recovery Readout (POST /api/gunny/recovery-readout) computes deterministic GO_HARD/NORMAL/DELOAD/REST recommendation from latest WearableConnection.syncData (recovery score, sleep duration, HRV, resting HR). Gunny generates the headline + guidance copy. Falls back to intake self-report when no wearable connected. Wearable enrichment also feeds chat — Gunny sees live recovery markers and dials intensity. Rendered in IntelCenter WEARABLES tab.</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2785,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="D72" s="40" t="inlineStr">
+      <c r="D72" s="59" t="inlineStr">
         <is>
           <t>LIVE</t>
         </is>
@@ -2781,30 +2797,22 @@
       </c>
       <c r="F72" s="38" t="inlineStr">
         <is>
-          <t>Gunny acknowledges in Spanish when language set to ES. Full TTS support.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
+          <t>Full app translation (142 keys per language) — not just Gunny acknowledgments. Persistent via localStorage (gunsup-language). Auto-detects browser language on first visit (navigator.language → ES). Updates document.documentElement.lang. Coverage: nav, login, dashboard, workout planner, IntelCenter tabs, billing, gunny, upgrade prompts, common copy. ES+EN switchable from header LanguageToggle.</t>
+        </is>
+      </c>
+    </row>
     <row r="82">
       <c r="A82" s="41" t="inlineStr">
         <is>
           <t>AUDIT</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="28" t="inlineStr">
         <is>
           <t>2026-04-27 audit confirmed all features verified live in code</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="28" t="inlineStr">
         <is>
           <t>Process</t>
         </is>
@@ -2814,12 +2822,12 @@
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="28" t="inlineStr">
         <is>
           <t>Tier gates 15/17/18/19/20/26/27/28/65 now enforced. Path engine #58 shipped. Wearable data flows to Gunny.</t>
         </is>
@@ -2838,240 +2846,240 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
+      <c r="A85" s="28" t="n">
         <v>69</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="28" t="inlineStr">
         <is>
           <t>Junior Operator account type (ages 10-18)</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
+      <c r="D85" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E85" s="28" t="inlineStr">
         <is>
           <t>Junior + Parent</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="28" t="inlineStr">
         <is>
           <t>isJunior flag + parentIds. Gated by JUNIOR_OPERATOR_ENABLED env.</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="n">
+      <c r="A86" s="28" t="n">
         <v>70</v>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="28" t="inlineStr">
         <is>
           <t>SOCCER_YOUTH_PROMPT (youth-safe Gunny)</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
+      <c r="D86" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E86" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="28" t="inlineStr">
         <is>
           <t>Replaces SYSTEM_PROMPT for juniors. Drops Marine DI, refers out concussion / RED-S / eating-disorder / supplements.</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="28" t="n">
         <v>71</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="28" t="inlineStr">
         <is>
           <t>JuniorIntakeForm (sport profile + parent consent)</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
+      <c r="D87" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E87" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="28" t="inlineStr">
         <is>
           <t>7-step youth-safe intake. No body-fat, no 1RM, no supplements. Parent consent gating.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="28" t="n">
         <v>72</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="28" t="inlineStr">
         <is>
           <t>Junior workload guardrails (Jayanthi / RPE / plyo caps)</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
+      <c r="D88" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E88" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="28" t="inlineStr">
         <is>
           <t>Server-side downscaler caps plyo contacts + RPE + session duration by maturation band.</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="28" t="n">
         <v>73</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="28" t="inlineStr">
         <is>
           <t>Junior safety event logger</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
+      <c r="D89" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E89" s="28" t="inlineStr">
         <is>
           <t>Junior + Parent</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" s="28" t="inlineStr">
         <is>
           <t>Pain / concussion / RED-S keyword detection. Persists to juniorSafety.events for parent dashboard.</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="n">
+      <c r="A90" s="28" t="n">
         <v>74</v>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="28" t="inlineStr">
         <is>
           <t>JuniorPRBoard (sport-performance metrics)</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
+      <c r="D90" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E90" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F90" s="28" t="inlineStr">
         <is>
           <t>14 metrics across speed/jump/agility/endurance/isometric. Replaces 1RM PRs for juniors.</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="n">
+      <c r="A91" s="28" t="n">
         <v>75</v>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="28" t="inlineStr">
         <is>
           <t>PARENT HUB tab</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="28" t="inlineStr">
         <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
+      <c r="D91" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E91" s="28" t="inlineStr">
         <is>
           <t>Parent (linked to junior)</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F91" s="28" t="inlineStr">
         <is>
           <t>Dedicated bottom-nav tab. Read-only training log, Gunny chat preview, safety events panel, emergency contact editor.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="n">
+      <c r="A92" s="28" t="n">
         <v>76</v>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="28" t="inlineStr">
         <is>
           <t>Youth research corpus (citation library)</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="28" t="inlineStr">
         <is>
           <t>Junior</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>LIVE</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
+      <c r="D92" s="28" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E92" s="28" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F92" s="28" t="inlineStr">
         <is>
           <t>docs/youth-soccer-corpus.md — 942 lines, 12 sections, 59 primary sources. Cited by SOCCER_YOUTH_PROMPT.</t>
         </is>
@@ -3583,10 +3591,10 @@
     <row r="17">
       <c r="A17" s="41" t="inlineStr">
         <is>
-          <t>UPDATED 2026-04-27</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+          <t>UPDATED 2026-04-26</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Prices reflect Stripe live mode + landing page</t>
         </is>

</xml_diff>

<commit_message>
docs(feature-report): mark #47 AI Form Analysis (Video) LIVE
Multi-frame video form review shipped — client-side frame
extraction + Claude vision returns structured JSON breakdown.
WARFIGHTER tier-gated. Rendered in IntelCenter FORM_CHECK tab.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/GUNS_UP_Feature_Report.xlsx
+++ b/docs/GUNS_UP_Feature_Report.xlsx
@@ -718,7 +718,7 @@
     <row r="1" ht="19.7" customHeight="1" s="29">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>Generated April 26, 2026 (post-build) — replaces April 27 audit version</t>
+          <t>Generated April 26, 2026 (post-build) — replaces April 27 audit version. Includes #47 Form Analysis (Video) build-out.</t>
         </is>
       </c>
     </row>
@@ -2155,9 +2155,9 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="D51" s="58" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+      <c r="D51" s="59" t="inlineStr">
+        <is>
+          <t>LIVE</t>
         </is>
       </c>
       <c r="E51" s="37" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="F51" s="38" t="inlineStr">
         <is>
-          <t>DEFERRED: Multi-frame video form analysis — corrections frame-by-frame. Photo Form Analysis (single image input) already LIVE via /api/gunny/analyze-form. Next session.</t>
+          <t>Multi-frame video form review (POST /api/gunny/analyze-form). Client extracts ~6 evenly-spaced keyframes from a clip via HTMLVideoElement+canvas (no server-side ffmpeg). Claude vision returns structured JSON: repsVisible, formScore (0-100), severity (green/yellow/red), per-phase breakdown (setup/descent/bottom/ascent/lockout), primaryFix, secondaryFixes, cuesToTry, safetyFlags (knee cave, lumbar flexion, bar drift), encouragement. Hard refusal for junior operators. Rendered in IntelCenter FORM_CHECK sub-tab. WARFIGHTER tier-gated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(feature-report): Pricing v2 + Activation + Food DB v2 LIVE
Three new feature rows added:
- Free RECON Tier (Pricing v2) — LIVE
- Post-Purchase Activation Flow — LIVE
- Food DB v2 (293 sourced entries) — LIVE

PRICING MODEL sheet RECON row updated to FREE with -$0.17/mo
platform loss reflecting Pricing Strategy v2 §3 unit economics
(intentional cost — funnel expansion).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/GUNS_UP_Feature_Report.xlsx
+++ b/docs/GUNS_UP_Feature_Report.xlsx
@@ -276,7 +276,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -451,6 +451,7 @@
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -718,7 +719,7 @@
     <row r="1" ht="19.7" customHeight="1" s="29">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>Generated April 26, 2026 (post-build) — replaces April 27 audit version. Includes #47 Form Analysis (Video) build-out.</t>
+          <t>Generated April 26, 2026 (post-build) — Pricing v2 + Activation Flow + Food DB v2 build-out. Supersedes April 27 audit.</t>
         </is>
       </c>
     </row>
@@ -729,6 +730,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="29">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -2801,6 +2803,102 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>77</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Free RECON Tier (Pricing v2)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="D73" s="60" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>All tiers</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>RECON dropped from $3.99/mo to FREE with hard rolling-window caps (30 chats/24h, 5 workout-gens/7d) enforced server-side via src/lib/usageCaps.ts. Paid tiers / admins / trainers bypass via OPS_CENTER_ACCESS check. Stripe checkout refuses tier=haiku. Landing page + BillingPanel reflect FREE with caps surfaced inline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>78</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Post-Purchase Activation Flow</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D74" s="60" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>COMMANDER+ (Stripe rail)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Bridge from Stripe checkout → app activation. AuthToken Prisma model + 9 activation tracking fields on Operator. POST /api/auth/web-handoff-token (iOS→web upgrade, 5min single-use). POST /api/auth/magic-link (send + consume; 7-day TTL). POST /api/auth/recover (3-strategy wizard: match / repair / support fallback). /welcome page polls checkout-session for tier. /recover page renders the wizard. 4-step activation email cadence (immediate/6h/3d/7d) via /api/cron/activation-emails (CRON_SECRET-protected). Stripe webhook fires Email 1 inline. Email provider wiring (Resend/Postmark) DEFERRED to next session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>79</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Food DB v2 (293 sourced entries)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Nutrition</t>
+        </is>
+      </c>
+      <c r="D75" s="60" t="inlineStr">
+        <is>
+          <t>LIVE</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>All tiers</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Replaces the implicit FOOD_DB string-keyed map with a structured 21-field schema covering 13 categories: Proteins (25), Grains (21), Fruits (15), Vegetables (15), Dairy (16), Fats/Nuts/Seeds (14), Legumes (10), Fast Food (49), Restaurant Staples (21), Latino/Mexican (37, ES names populated), Supplements (23), Condiments (21), Beverages (26). Sources: USDA FoodData Central, official chain nutrition guides, manufacturer labels, ISSN position stands, NIH ODS fact sheets. Wired into Gunny system prompt + dynamic message-aware injection (id-match → component reconstruct → estimate fallback).</t>
+        </is>
+      </c>
+    </row>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
     <row r="82">
       <c r="A82" s="41" t="inlineStr">
         <is>
@@ -2833,6 +2931,7 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
     <row r="84">
       <c r="A84" s="42" t="inlineStr">
         <is>
@@ -3200,31 +3299,33 @@
         </is>
       </c>
       <c r="D4" s="45" t="n">
-        <v>3.99</v>
+        <v>0</v>
       </c>
       <c r="E4" s="45" t="n">
-        <v>39.92</v>
+        <v>0</v>
       </c>
       <c r="F4" s="45" t="n">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="G4" s="45" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="H4" s="45" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="I4" s="45" t="n">
         <v>0.1</v>
       </c>
       <c r="J4" s="45" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K4" s="45" t="n">
-        <v>2.96</v>
-      </c>
-      <c r="L4" s="46" t="n">
-        <v>0.742</v>
+        <v>-0.17</v>
+      </c>
+      <c r="L4" s="46" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="29">
@@ -3591,12 +3692,12 @@
     <row r="17">
       <c r="A17" s="41" t="inlineStr">
         <is>
-          <t>UPDATED 2026-04-26</t>
+          <t>UPDATED 2026-04-26 — Pricing v2 (RECON FREE)</t>
         </is>
       </c>
       <c r="B17" s="28" t="inlineStr">
         <is>
-          <t>Prices reflect Stripe live mode + landing page</t>
+          <t>Prices reflect Pricing Strategy v2 + Stripe live mode</t>
         </is>
       </c>
     </row>

</xml_diff>